<commit_message>
máy chủ: tên tướng/vật phẩm/bí kíp/hồn ngọc/thần khí/sưu tập theo client
Cổng GM (và mọi chữ máy chủ tự phát: thư, thông báo) gọi tên theo bộ Excel của một bản game
khác (kiếm hiệp: "Trương Vô Kỵ", "Tửu Túy Quyền", "Đan tiến giai") trong khi người chơi
thấy One Piece. Đã quyết client là đúng, nên máy chủ theo client.

- tools/dong-bo-ten-server.py: ghi đè cột tên/目标文本 của 文本库, 装备表, 符文基础, 命格基础,
  仙器基础, 仙器碎片, 藏品基础 trong excel-src và 基础物品/碎片 thẳng trong XML của
  item-table.xlsm (ô công thức -> hằng số); chỉ id có ở cả hai bên.
- 6 workbook biên dịch lại từ JSON, 7 file qua ExcelProbe (parser thật, JDK 8 trong Docker).
- Danh mục cổng GM sinh lại (6588 mục, cùng tên với kho đồ console trả).
- Ghi nhận: excel/reload trên cụm này làm JVM game OOM -> restart container thay vì reload.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/server/excel/release/rune.xlsx
+++ b/server/excel/release/rune.xlsx
@@ -616,7 +616,7 @@
     <t xml:space="preserve">估值</t>
   </si>
   <si>
-    <t xml:space="preserve">Tửu Túy Quyền</t>
+    <t xml:space="preserve">Haki cấp 1</t>
   </si>
   <si>
     <t xml:space="preserve">Cường hóa tướng</t>
@@ -640,7 +640,7 @@
     <t xml:space="preserve">3:100004:60</t>
   </si>
   <si>
-    <t xml:space="preserve">Thái Cực Kiếm</t>
+    <t xml:space="preserve">Haki cấp 2</t>
   </si>
   <si>
     <t xml:space="preserve">1:10000</t>
@@ -658,7 +658,7 @@
     <t xml:space="preserve">3:100004:300</t>
   </si>
   <si>
-    <t xml:space="preserve">Cửu Âm Công</t>
+    <t xml:space="preserve">Haki cấp 3</t>
   </si>
   <si>
     <t xml:space="preserve">1,1:3000#1,2:3000#2:4000</t>
@@ -679,7 +679,7 @@
     <t xml:space="preserve">3:100004:1500</t>
   </si>
   <si>
-    <t xml:space="preserve">Nhất Chỉ Công</t>
+    <t xml:space="preserve">Haki cấp S</t>
   </si>
   <si>
     <t xml:space="preserve">3,2:3000#3,1:3000#2,2:2000#3,2:2000</t>
@@ -706,7 +706,7 @@
     <t xml:space="preserve">3:100004:7500</t>
   </si>
   <si>
-    <t xml:space="preserve">Cửu Dương Công</t>
+    <t xml:space="preserve">Haki cấp SS</t>
   </si>
   <si>
     <t xml:space="preserve">5,6</t>
@@ -733,7 +733,7 @@
     <t xml:space="preserve">3:100004:37500</t>
   </si>
   <si>
-    <t xml:space="preserve">Thiên Ngoại Phi Tiên</t>
+    <t xml:space="preserve">Haki cấp SSS</t>
   </si>
   <si>
     <t xml:space="preserve">2#1</t>
@@ -853,7 +853,7 @@
     <t xml:space="preserve">3:100004:10000#0:0:2000000</t>
   </si>
   <si>
-    <t xml:space="preserve">Sách thiên phú</t>
+    <t xml:space="preserve">Năng Lượng Haki</t>
   </si>
   <si>
     <t xml:space="preserve">技能等级组合</t>

</xml_diff>